<commit_message>
Base de donnees remplisaage debut
</commit_message>
<xml_diff>
--- a/Planning de la semaine/Semaine_27_juillet_au _01_aout_2026.xlsx
+++ b/Planning de la semaine/Semaine_27_juillet_au _01_aout_2026.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\NextOri\Planning de la semaine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{110D8B6A-A601-457D-8A6B-9C6EBF1AD075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{151B9234-B84C-43B9-B536-D588E1B001FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{149C7D14-FD66-4BB6-9593-C9A067902534}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{149C7D14-FD66-4BB6-9593-C9A067902534}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="Feuil 2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="31">
   <si>
     <t>Lundi</t>
   </si>
@@ -100,6 +101,24 @@
   </si>
   <si>
     <t>MASSOYA</t>
+  </si>
+  <si>
+    <t>Planning de la semaine du 03/08/2026 au 09/08/2026</t>
+  </si>
+  <si>
+    <t>Completer la base de donnees des metiers, filieres et universites</t>
+  </si>
+  <si>
+    <t>Gestion des favoris et historiques</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestion des series de connexion et elargissement calcul de points et de badges </t>
+  </si>
+  <si>
+    <t>Debut page Dashboard Admin</t>
+  </si>
+  <si>
+    <t>Fin prevu de la page Dashboard Admin</t>
   </si>
 </sst>
 </file>
@@ -141,14 +160,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -173,8 +194,24 @@
     <tableColumn id="2" xr3:uid="{3F409BE1-FE7A-4BF9-B86B-9AFFF638C21A}" name="Taches"/>
     <tableColumn id="3" xr3:uid="{5FDCAA10-02BF-4111-95A6-2647F2F13D00}" name="Debut/h"/>
     <tableColumn id="4" xr3:uid="{F37070A9-060A-4EBF-A049-73AF8CEED0D8}" name="Fin/h"/>
-    <tableColumn id="5" xr3:uid="{0154D75D-FDEB-47F3-BE13-E55FB442A6D9}" name="Duree/h" dataDxfId="0">
+    <tableColumn id="5" xr3:uid="{0154D75D-FDEB-47F3-BE13-E55FB442A6D9}" name="Duree/h" dataDxfId="1">
       <calculatedColumnFormula>Tableau1[[#This Row],[Fin/h]]-Tableau1[[#This Row],[Debut/h]]</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2045620D-21AC-46EA-8769-D8D21BD8BC54}" name="Tableau13" displayName="Tableau13" ref="B2:F10" totalsRowShown="0">
+  <autoFilter ref="B2:F10" xr:uid="{2EC4B212-B6D0-4E43-A56C-37D94FFF9C11}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{47A016C0-F158-4BEE-8572-11220636706E}" name="Date"/>
+    <tableColumn id="2" xr3:uid="{ECBBB647-29EF-4D0C-8ED4-7312B8FB94F6}" name="Taches"/>
+    <tableColumn id="3" xr3:uid="{3E0B87A4-D1A7-4D70-9C5B-0267AEDAB739}" name="Debut/h"/>
+    <tableColumn id="4" xr3:uid="{4545CED6-857E-4B74-AC2C-3D6BA5B7E04E}" name="Fin/h"/>
+    <tableColumn id="5" xr3:uid="{59F0DDFD-B50B-4BF3-9E22-57E02A15D5B8}" name="Duree/h" dataDxfId="0">
+      <calculatedColumnFormula>Tableau13[[#This Row],[Fin/h]]-Tableau13[[#This Row],[Debut/h]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -514,7 +551,7 @@
       <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3">
         <v>15</v>
       </c>
       <c r="E3">
@@ -532,7 +569,7 @@
       <c r="C4" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4">
         <v>15</v>
       </c>
       <c r="E4">
@@ -550,7 +587,7 @@
       <c r="C5" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5">
         <v>15</v>
       </c>
       <c r="E5">
@@ -630,7 +667,7 @@
       <c r="E10" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10">
         <f>SUBTOTAL(109,F3:F9)</f>
         <v>30</v>
       </c>
@@ -660,4 +697,189 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C6A26B7-7AF8-4FB8-8B0F-C59B9A0B51E1}">
+  <dimension ref="B1:F15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="73.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3">
+        <v>10</v>
+      </c>
+      <c r="E3">
+        <v>19</v>
+      </c>
+      <c r="F3">
+        <f>Tableau13[[#This Row],[Fin/h]]-Tableau13[[#This Row],[Debut/h]]</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4">
+        <v>15</v>
+      </c>
+      <c r="E4">
+        <v>20</v>
+      </c>
+      <c r="F4">
+        <f>Tableau13[[#This Row],[Fin/h]]-Tableau13[[#This Row],[Debut/h]]</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5">
+        <v>15</v>
+      </c>
+      <c r="E5">
+        <v>20</v>
+      </c>
+      <c r="F5">
+        <f>Tableau13[[#This Row],[Fin/h]]-Tableau13[[#This Row],[Debut/h]]</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7">
+        <v>18</v>
+      </c>
+      <c r="E7">
+        <v>20</v>
+      </c>
+      <c r="F7">
+        <f>Tableau13[[#This Row],[Fin/h]]-Tableau13[[#This Row],[Debut/h]]</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8">
+        <v>15</v>
+      </c>
+      <c r="E8">
+        <v>20</v>
+      </c>
+      <c r="F8">
+        <f>Tableau13[[#This Row],[Fin/h]]-Tableau13[[#This Row],[Debut/h]]</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9">
+        <v>17</v>
+      </c>
+      <c r="E9">
+        <v>20</v>
+      </c>
+      <c r="F9">
+        <f>Tableau13[[#This Row],[Fin/h]]-Tableau13[[#This Row],[Debut/h]]</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10">
+        <f>SUBTOTAL(109,F3:F9)</f>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="F14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="F15" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>